<commit_message>
Smart Revision part 2: "Recommended for you" offers matched to weak topics
- Migration: revision_offers + revision_offer_sections (staff-only RLS),
  apply_revision_offers (import job), consent-gated my_revision_offers
- Offers sheet in the timetable spreadsheet (topic + sub-topic numbers)
- Revision Home card: up to 2 offers covering the student's weak sub-topics,
  no price or payment; "ask your parent or the centre"
- ADR 0010 records the owner's decision; CLAUDE.md PDPA line updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EdB7jr7dZB3nArHF8Gftsp
</commit_message>
<xml_diff>
--- a/docs/templates/timetable-template.xlsx
+++ b/docs/templates/timetable-template.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancellations" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exams" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offers" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -651,19 +652,50 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
+          <t>Offers</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Programmes to recommend in Smart Revision → "Recommended for you", e.g. P6 | Science | Holiday Intensive | Four extra lessons in December | Energy | 1, 3 | 1/11/2026 | 15/12/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Topic is a question bank topic for that course; Sub-topics are its section numbers (leave blank for the whole topic). A student sees an offer only when one of those sub-topics is weak for them AND their guardian gave marketing consent. Students never see a price or a way to pay: they are told to ask a parent or the centre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Listing a course's offers replaces that course's offers; leave the sheet empty to keep them. From / Until date are optional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
           <t>Example (Classes)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>P5MA-SAT-0900 | P5 | Mathematics | Physical tutorial | Bishan | Room 1 | Ms Lim | Sat | 09:00 | 120 | 3/1/2027 | 30/12/2027 | 12 |</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>P6SC-WED-LIVE | P6 | Science | Live tutorial | | | Mr Ong | Wed | 19:30 | 90 | 6/1/2027 | 29/12/2027 | | https://zoom.us/j/123456789</t>
         </is>
@@ -12034,4 +12066,2066 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H500"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Sub-topics</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>From date</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Until date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+    </row>
+    <row r="3">
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="G19" s="5" t="n"/>
+      <c r="H19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="G26" s="5" t="n"/>
+      <c r="H26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="G34" s="5" t="n"/>
+      <c r="H34" s="5" t="n"/>
+    </row>
+    <row r="35">
+      <c r="G35" s="5" t="n"/>
+      <c r="H35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="5" t="n"/>
+    </row>
+    <row r="37">
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="5" t="n"/>
+    </row>
+    <row r="39">
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="5" t="n"/>
+    </row>
+    <row r="41">
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="5" t="n"/>
+    </row>
+    <row r="43">
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="G44" s="5" t="n"/>
+      <c r="H44" s="5" t="n"/>
+    </row>
+    <row r="45">
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="G46" s="5" t="n"/>
+      <c r="H46" s="5" t="n"/>
+    </row>
+    <row r="47">
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="G48" s="5" t="n"/>
+      <c r="H48" s="5" t="n"/>
+    </row>
+    <row r="49">
+      <c r="G49" s="5" t="n"/>
+      <c r="H49" s="5" t="n"/>
+    </row>
+    <row r="50">
+      <c r="G50" s="5" t="n"/>
+      <c r="H50" s="5" t="n"/>
+    </row>
+    <row r="51">
+      <c r="G51" s="5" t="n"/>
+      <c r="H51" s="5" t="n"/>
+    </row>
+    <row r="52">
+      <c r="G52" s="5" t="n"/>
+      <c r="H52" s="5" t="n"/>
+    </row>
+    <row r="53">
+      <c r="G53" s="5" t="n"/>
+      <c r="H53" s="5" t="n"/>
+    </row>
+    <row r="54">
+      <c r="G54" s="5" t="n"/>
+      <c r="H54" s="5" t="n"/>
+    </row>
+    <row r="55">
+      <c r="G55" s="5" t="n"/>
+      <c r="H55" s="5" t="n"/>
+    </row>
+    <row r="56">
+      <c r="G56" s="5" t="n"/>
+      <c r="H56" s="5" t="n"/>
+    </row>
+    <row r="57">
+      <c r="G57" s="5" t="n"/>
+      <c r="H57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="G58" s="5" t="n"/>
+      <c r="H58" s="5" t="n"/>
+    </row>
+    <row r="59">
+      <c r="G59" s="5" t="n"/>
+      <c r="H59" s="5" t="n"/>
+    </row>
+    <row r="60">
+      <c r="G60" s="5" t="n"/>
+      <c r="H60" s="5" t="n"/>
+    </row>
+    <row r="61">
+      <c r="G61" s="5" t="n"/>
+      <c r="H61" s="5" t="n"/>
+    </row>
+    <row r="62">
+      <c r="G62" s="5" t="n"/>
+      <c r="H62" s="5" t="n"/>
+    </row>
+    <row r="63">
+      <c r="G63" s="5" t="n"/>
+      <c r="H63" s="5" t="n"/>
+    </row>
+    <row r="64">
+      <c r="G64" s="5" t="n"/>
+      <c r="H64" s="5" t="n"/>
+    </row>
+    <row r="65">
+      <c r="G65" s="5" t="n"/>
+      <c r="H65" s="5" t="n"/>
+    </row>
+    <row r="66">
+      <c r="G66" s="5" t="n"/>
+      <c r="H66" s="5" t="n"/>
+    </row>
+    <row r="67">
+      <c r="G67" s="5" t="n"/>
+      <c r="H67" s="5" t="n"/>
+    </row>
+    <row r="68">
+      <c r="G68" s="5" t="n"/>
+      <c r="H68" s="5" t="n"/>
+    </row>
+    <row r="69">
+      <c r="G69" s="5" t="n"/>
+      <c r="H69" s="5" t="n"/>
+    </row>
+    <row r="70">
+      <c r="G70" s="5" t="n"/>
+      <c r="H70" s="5" t="n"/>
+    </row>
+    <row r="71">
+      <c r="G71" s="5" t="n"/>
+      <c r="H71" s="5" t="n"/>
+    </row>
+    <row r="72">
+      <c r="G72" s="5" t="n"/>
+      <c r="H72" s="5" t="n"/>
+    </row>
+    <row r="73">
+      <c r="G73" s="5" t="n"/>
+      <c r="H73" s="5" t="n"/>
+    </row>
+    <row r="74">
+      <c r="G74" s="5" t="n"/>
+      <c r="H74" s="5" t="n"/>
+    </row>
+    <row r="75">
+      <c r="G75" s="5" t="n"/>
+      <c r="H75" s="5" t="n"/>
+    </row>
+    <row r="76">
+      <c r="G76" s="5" t="n"/>
+      <c r="H76" s="5" t="n"/>
+    </row>
+    <row r="77">
+      <c r="G77" s="5" t="n"/>
+      <c r="H77" s="5" t="n"/>
+    </row>
+    <row r="78">
+      <c r="G78" s="5" t="n"/>
+      <c r="H78" s="5" t="n"/>
+    </row>
+    <row r="79">
+      <c r="G79" s="5" t="n"/>
+      <c r="H79" s="5" t="n"/>
+    </row>
+    <row r="80">
+      <c r="G80" s="5" t="n"/>
+      <c r="H80" s="5" t="n"/>
+    </row>
+    <row r="81">
+      <c r="G81" s="5" t="n"/>
+      <c r="H81" s="5" t="n"/>
+    </row>
+    <row r="82">
+      <c r="G82" s="5" t="n"/>
+      <c r="H82" s="5" t="n"/>
+    </row>
+    <row r="83">
+      <c r="G83" s="5" t="n"/>
+      <c r="H83" s="5" t="n"/>
+    </row>
+    <row r="84">
+      <c r="G84" s="5" t="n"/>
+      <c r="H84" s="5" t="n"/>
+    </row>
+    <row r="85">
+      <c r="G85" s="5" t="n"/>
+      <c r="H85" s="5" t="n"/>
+    </row>
+    <row r="86">
+      <c r="G86" s="5" t="n"/>
+      <c r="H86" s="5" t="n"/>
+    </row>
+    <row r="87">
+      <c r="G87" s="5" t="n"/>
+      <c r="H87" s="5" t="n"/>
+    </row>
+    <row r="88">
+      <c r="G88" s="5" t="n"/>
+      <c r="H88" s="5" t="n"/>
+    </row>
+    <row r="89">
+      <c r="G89" s="5" t="n"/>
+      <c r="H89" s="5" t="n"/>
+    </row>
+    <row r="90">
+      <c r="G90" s="5" t="n"/>
+      <c r="H90" s="5" t="n"/>
+    </row>
+    <row r="91">
+      <c r="G91" s="5" t="n"/>
+      <c r="H91" s="5" t="n"/>
+    </row>
+    <row r="92">
+      <c r="G92" s="5" t="n"/>
+      <c r="H92" s="5" t="n"/>
+    </row>
+    <row r="93">
+      <c r="G93" s="5" t="n"/>
+      <c r="H93" s="5" t="n"/>
+    </row>
+    <row r="94">
+      <c r="G94" s="5" t="n"/>
+      <c r="H94" s="5" t="n"/>
+    </row>
+    <row r="95">
+      <c r="G95" s="5" t="n"/>
+      <c r="H95" s="5" t="n"/>
+    </row>
+    <row r="96">
+      <c r="G96" s="5" t="n"/>
+      <c r="H96" s="5" t="n"/>
+    </row>
+    <row r="97">
+      <c r="G97" s="5" t="n"/>
+      <c r="H97" s="5" t="n"/>
+    </row>
+    <row r="98">
+      <c r="G98" s="5" t="n"/>
+      <c r="H98" s="5" t="n"/>
+    </row>
+    <row r="99">
+      <c r="G99" s="5" t="n"/>
+      <c r="H99" s="5" t="n"/>
+    </row>
+    <row r="100">
+      <c r="G100" s="5" t="n"/>
+      <c r="H100" s="5" t="n"/>
+    </row>
+    <row r="101">
+      <c r="G101" s="5" t="n"/>
+      <c r="H101" s="5" t="n"/>
+    </row>
+    <row r="102">
+      <c r="G102" s="5" t="n"/>
+      <c r="H102" s="5" t="n"/>
+    </row>
+    <row r="103">
+      <c r="G103" s="5" t="n"/>
+      <c r="H103" s="5" t="n"/>
+    </row>
+    <row r="104">
+      <c r="G104" s="5" t="n"/>
+      <c r="H104" s="5" t="n"/>
+    </row>
+    <row r="105">
+      <c r="G105" s="5" t="n"/>
+      <c r="H105" s="5" t="n"/>
+    </row>
+    <row r="106">
+      <c r="G106" s="5" t="n"/>
+      <c r="H106" s="5" t="n"/>
+    </row>
+    <row r="107">
+      <c r="G107" s="5" t="n"/>
+      <c r="H107" s="5" t="n"/>
+    </row>
+    <row r="108">
+      <c r="G108" s="5" t="n"/>
+      <c r="H108" s="5" t="n"/>
+    </row>
+    <row r="109">
+      <c r="G109" s="5" t="n"/>
+      <c r="H109" s="5" t="n"/>
+    </row>
+    <row r="110">
+      <c r="G110" s="5" t="n"/>
+      <c r="H110" s="5" t="n"/>
+    </row>
+    <row r="111">
+      <c r="G111" s="5" t="n"/>
+      <c r="H111" s="5" t="n"/>
+    </row>
+    <row r="112">
+      <c r="G112" s="5" t="n"/>
+      <c r="H112" s="5" t="n"/>
+    </row>
+    <row r="113">
+      <c r="G113" s="5" t="n"/>
+      <c r="H113" s="5" t="n"/>
+    </row>
+    <row r="114">
+      <c r="G114" s="5" t="n"/>
+      <c r="H114" s="5" t="n"/>
+    </row>
+    <row r="115">
+      <c r="G115" s="5" t="n"/>
+      <c r="H115" s="5" t="n"/>
+    </row>
+    <row r="116">
+      <c r="G116" s="5" t="n"/>
+      <c r="H116" s="5" t="n"/>
+    </row>
+    <row r="117">
+      <c r="G117" s="5" t="n"/>
+      <c r="H117" s="5" t="n"/>
+    </row>
+    <row r="118">
+      <c r="G118" s="5" t="n"/>
+      <c r="H118" s="5" t="n"/>
+    </row>
+    <row r="119">
+      <c r="G119" s="5" t="n"/>
+      <c r="H119" s="5" t="n"/>
+    </row>
+    <row r="120">
+      <c r="G120" s="5" t="n"/>
+      <c r="H120" s="5" t="n"/>
+    </row>
+    <row r="121">
+      <c r="G121" s="5" t="n"/>
+      <c r="H121" s="5" t="n"/>
+    </row>
+    <row r="122">
+      <c r="G122" s="5" t="n"/>
+      <c r="H122" s="5" t="n"/>
+    </row>
+    <row r="123">
+      <c r="G123" s="5" t="n"/>
+      <c r="H123" s="5" t="n"/>
+    </row>
+    <row r="124">
+      <c r="G124" s="5" t="n"/>
+      <c r="H124" s="5" t="n"/>
+    </row>
+    <row r="125">
+      <c r="G125" s="5" t="n"/>
+      <c r="H125" s="5" t="n"/>
+    </row>
+    <row r="126">
+      <c r="G126" s="5" t="n"/>
+      <c r="H126" s="5" t="n"/>
+    </row>
+    <row r="127">
+      <c r="G127" s="5" t="n"/>
+      <c r="H127" s="5" t="n"/>
+    </row>
+    <row r="128">
+      <c r="G128" s="5" t="n"/>
+      <c r="H128" s="5" t="n"/>
+    </row>
+    <row r="129">
+      <c r="G129" s="5" t="n"/>
+      <c r="H129" s="5" t="n"/>
+    </row>
+    <row r="130">
+      <c r="G130" s="5" t="n"/>
+      <c r="H130" s="5" t="n"/>
+    </row>
+    <row r="131">
+      <c r="G131" s="5" t="n"/>
+      <c r="H131" s="5" t="n"/>
+    </row>
+    <row r="132">
+      <c r="G132" s="5" t="n"/>
+      <c r="H132" s="5" t="n"/>
+    </row>
+    <row r="133">
+      <c r="G133" s="5" t="n"/>
+      <c r="H133" s="5" t="n"/>
+    </row>
+    <row r="134">
+      <c r="G134" s="5" t="n"/>
+      <c r="H134" s="5" t="n"/>
+    </row>
+    <row r="135">
+      <c r="G135" s="5" t="n"/>
+      <c r="H135" s="5" t="n"/>
+    </row>
+    <row r="136">
+      <c r="G136" s="5" t="n"/>
+      <c r="H136" s="5" t="n"/>
+    </row>
+    <row r="137">
+      <c r="G137" s="5" t="n"/>
+      <c r="H137" s="5" t="n"/>
+    </row>
+    <row r="138">
+      <c r="G138" s="5" t="n"/>
+      <c r="H138" s="5" t="n"/>
+    </row>
+    <row r="139">
+      <c r="G139" s="5" t="n"/>
+      <c r="H139" s="5" t="n"/>
+    </row>
+    <row r="140">
+      <c r="G140" s="5" t="n"/>
+      <c r="H140" s="5" t="n"/>
+    </row>
+    <row r="141">
+      <c r="G141" s="5" t="n"/>
+      <c r="H141" s="5" t="n"/>
+    </row>
+    <row r="142">
+      <c r="G142" s="5" t="n"/>
+      <c r="H142" s="5" t="n"/>
+    </row>
+    <row r="143">
+      <c r="G143" s="5" t="n"/>
+      <c r="H143" s="5" t="n"/>
+    </row>
+    <row r="144">
+      <c r="G144" s="5" t="n"/>
+      <c r="H144" s="5" t="n"/>
+    </row>
+    <row r="145">
+      <c r="G145" s="5" t="n"/>
+      <c r="H145" s="5" t="n"/>
+    </row>
+    <row r="146">
+      <c r="G146" s="5" t="n"/>
+      <c r="H146" s="5" t="n"/>
+    </row>
+    <row r="147">
+      <c r="G147" s="5" t="n"/>
+      <c r="H147" s="5" t="n"/>
+    </row>
+    <row r="148">
+      <c r="G148" s="5" t="n"/>
+      <c r="H148" s="5" t="n"/>
+    </row>
+    <row r="149">
+      <c r="G149" s="5" t="n"/>
+      <c r="H149" s="5" t="n"/>
+    </row>
+    <row r="150">
+      <c r="G150" s="5" t="n"/>
+      <c r="H150" s="5" t="n"/>
+    </row>
+    <row r="151">
+      <c r="G151" s="5" t="n"/>
+      <c r="H151" s="5" t="n"/>
+    </row>
+    <row r="152">
+      <c r="G152" s="5" t="n"/>
+      <c r="H152" s="5" t="n"/>
+    </row>
+    <row r="153">
+      <c r="G153" s="5" t="n"/>
+      <c r="H153" s="5" t="n"/>
+    </row>
+    <row r="154">
+      <c r="G154" s="5" t="n"/>
+      <c r="H154" s="5" t="n"/>
+    </row>
+    <row r="155">
+      <c r="G155" s="5" t="n"/>
+      <c r="H155" s="5" t="n"/>
+    </row>
+    <row r="156">
+      <c r="G156" s="5" t="n"/>
+      <c r="H156" s="5" t="n"/>
+    </row>
+    <row r="157">
+      <c r="G157" s="5" t="n"/>
+      <c r="H157" s="5" t="n"/>
+    </row>
+    <row r="158">
+      <c r="G158" s="5" t="n"/>
+      <c r="H158" s="5" t="n"/>
+    </row>
+    <row r="159">
+      <c r="G159" s="5" t="n"/>
+      <c r="H159" s="5" t="n"/>
+    </row>
+    <row r="160">
+      <c r="G160" s="5" t="n"/>
+      <c r="H160" s="5" t="n"/>
+    </row>
+    <row r="161">
+      <c r="G161" s="5" t="n"/>
+      <c r="H161" s="5" t="n"/>
+    </row>
+    <row r="162">
+      <c r="G162" s="5" t="n"/>
+      <c r="H162" s="5" t="n"/>
+    </row>
+    <row r="163">
+      <c r="G163" s="5" t="n"/>
+      <c r="H163" s="5" t="n"/>
+    </row>
+    <row r="164">
+      <c r="G164" s="5" t="n"/>
+      <c r="H164" s="5" t="n"/>
+    </row>
+    <row r="165">
+      <c r="G165" s="5" t="n"/>
+      <c r="H165" s="5" t="n"/>
+    </row>
+    <row r="166">
+      <c r="G166" s="5" t="n"/>
+      <c r="H166" s="5" t="n"/>
+    </row>
+    <row r="167">
+      <c r="G167" s="5" t="n"/>
+      <c r="H167" s="5" t="n"/>
+    </row>
+    <row r="168">
+      <c r="G168" s="5" t="n"/>
+      <c r="H168" s="5" t="n"/>
+    </row>
+    <row r="169">
+      <c r="G169" s="5" t="n"/>
+      <c r="H169" s="5" t="n"/>
+    </row>
+    <row r="170">
+      <c r="G170" s="5" t="n"/>
+      <c r="H170" s="5" t="n"/>
+    </row>
+    <row r="171">
+      <c r="G171" s="5" t="n"/>
+      <c r="H171" s="5" t="n"/>
+    </row>
+    <row r="172">
+      <c r="G172" s="5" t="n"/>
+      <c r="H172" s="5" t="n"/>
+    </row>
+    <row r="173">
+      <c r="G173" s="5" t="n"/>
+      <c r="H173" s="5" t="n"/>
+    </row>
+    <row r="174">
+      <c r="G174" s="5" t="n"/>
+      <c r="H174" s="5" t="n"/>
+    </row>
+    <row r="175">
+      <c r="G175" s="5" t="n"/>
+      <c r="H175" s="5" t="n"/>
+    </row>
+    <row r="176">
+      <c r="G176" s="5" t="n"/>
+      <c r="H176" s="5" t="n"/>
+    </row>
+    <row r="177">
+      <c r="G177" s="5" t="n"/>
+      <c r="H177" s="5" t="n"/>
+    </row>
+    <row r="178">
+      <c r="G178" s="5" t="n"/>
+      <c r="H178" s="5" t="n"/>
+    </row>
+    <row r="179">
+      <c r="G179" s="5" t="n"/>
+      <c r="H179" s="5" t="n"/>
+    </row>
+    <row r="180">
+      <c r="G180" s="5" t="n"/>
+      <c r="H180" s="5" t="n"/>
+    </row>
+    <row r="181">
+      <c r="G181" s="5" t="n"/>
+      <c r="H181" s="5" t="n"/>
+    </row>
+    <row r="182">
+      <c r="G182" s="5" t="n"/>
+      <c r="H182" s="5" t="n"/>
+    </row>
+    <row r="183">
+      <c r="G183" s="5" t="n"/>
+      <c r="H183" s="5" t="n"/>
+    </row>
+    <row r="184">
+      <c r="G184" s="5" t="n"/>
+      <c r="H184" s="5" t="n"/>
+    </row>
+    <row r="185">
+      <c r="G185" s="5" t="n"/>
+      <c r="H185" s="5" t="n"/>
+    </row>
+    <row r="186">
+      <c r="G186" s="5" t="n"/>
+      <c r="H186" s="5" t="n"/>
+    </row>
+    <row r="187">
+      <c r="G187" s="5" t="n"/>
+      <c r="H187" s="5" t="n"/>
+    </row>
+    <row r="188">
+      <c r="G188" s="5" t="n"/>
+      <c r="H188" s="5" t="n"/>
+    </row>
+    <row r="189">
+      <c r="G189" s="5" t="n"/>
+      <c r="H189" s="5" t="n"/>
+    </row>
+    <row r="190">
+      <c r="G190" s="5" t="n"/>
+      <c r="H190" s="5" t="n"/>
+    </row>
+    <row r="191">
+      <c r="G191" s="5" t="n"/>
+      <c r="H191" s="5" t="n"/>
+    </row>
+    <row r="192">
+      <c r="G192" s="5" t="n"/>
+      <c r="H192" s="5" t="n"/>
+    </row>
+    <row r="193">
+      <c r="G193" s="5" t="n"/>
+      <c r="H193" s="5" t="n"/>
+    </row>
+    <row r="194">
+      <c r="G194" s="5" t="n"/>
+      <c r="H194" s="5" t="n"/>
+    </row>
+    <row r="195">
+      <c r="G195" s="5" t="n"/>
+      <c r="H195" s="5" t="n"/>
+    </row>
+    <row r="196">
+      <c r="G196" s="5" t="n"/>
+      <c r="H196" s="5" t="n"/>
+    </row>
+    <row r="197">
+      <c r="G197" s="5" t="n"/>
+      <c r="H197" s="5" t="n"/>
+    </row>
+    <row r="198">
+      <c r="G198" s="5" t="n"/>
+      <c r="H198" s="5" t="n"/>
+    </row>
+    <row r="199">
+      <c r="G199" s="5" t="n"/>
+      <c r="H199" s="5" t="n"/>
+    </row>
+    <row r="200">
+      <c r="G200" s="5" t="n"/>
+      <c r="H200" s="5" t="n"/>
+    </row>
+    <row r="201">
+      <c r="G201" s="5" t="n"/>
+      <c r="H201" s="5" t="n"/>
+    </row>
+    <row r="202">
+      <c r="G202" s="5" t="n"/>
+      <c r="H202" s="5" t="n"/>
+    </row>
+    <row r="203">
+      <c r="G203" s="5" t="n"/>
+      <c r="H203" s="5" t="n"/>
+    </row>
+    <row r="204">
+      <c r="G204" s="5" t="n"/>
+      <c r="H204" s="5" t="n"/>
+    </row>
+    <row r="205">
+      <c r="G205" s="5" t="n"/>
+      <c r="H205" s="5" t="n"/>
+    </row>
+    <row r="206">
+      <c r="G206" s="5" t="n"/>
+      <c r="H206" s="5" t="n"/>
+    </row>
+    <row r="207">
+      <c r="G207" s="5" t="n"/>
+      <c r="H207" s="5" t="n"/>
+    </row>
+    <row r="208">
+      <c r="G208" s="5" t="n"/>
+      <c r="H208" s="5" t="n"/>
+    </row>
+    <row r="209">
+      <c r="G209" s="5" t="n"/>
+      <c r="H209" s="5" t="n"/>
+    </row>
+    <row r="210">
+      <c r="G210" s="5" t="n"/>
+      <c r="H210" s="5" t="n"/>
+    </row>
+    <row r="211">
+      <c r="G211" s="5" t="n"/>
+      <c r="H211" s="5" t="n"/>
+    </row>
+    <row r="212">
+      <c r="G212" s="5" t="n"/>
+      <c r="H212" s="5" t="n"/>
+    </row>
+    <row r="213">
+      <c r="G213" s="5" t="n"/>
+      <c r="H213" s="5" t="n"/>
+    </row>
+    <row r="214">
+      <c r="G214" s="5" t="n"/>
+      <c r="H214" s="5" t="n"/>
+    </row>
+    <row r="215">
+      <c r="G215" s="5" t="n"/>
+      <c r="H215" s="5" t="n"/>
+    </row>
+    <row r="216">
+      <c r="G216" s="5" t="n"/>
+      <c r="H216" s="5" t="n"/>
+    </row>
+    <row r="217">
+      <c r="G217" s="5" t="n"/>
+      <c r="H217" s="5" t="n"/>
+    </row>
+    <row r="218">
+      <c r="G218" s="5" t="n"/>
+      <c r="H218" s="5" t="n"/>
+    </row>
+    <row r="219">
+      <c r="G219" s="5" t="n"/>
+      <c r="H219" s="5" t="n"/>
+    </row>
+    <row r="220">
+      <c r="G220" s="5" t="n"/>
+      <c r="H220" s="5" t="n"/>
+    </row>
+    <row r="221">
+      <c r="G221" s="5" t="n"/>
+      <c r="H221" s="5" t="n"/>
+    </row>
+    <row r="222">
+      <c r="G222" s="5" t="n"/>
+      <c r="H222" s="5" t="n"/>
+    </row>
+    <row r="223">
+      <c r="G223" s="5" t="n"/>
+      <c r="H223" s="5" t="n"/>
+    </row>
+    <row r="224">
+      <c r="G224" s="5" t="n"/>
+      <c r="H224" s="5" t="n"/>
+    </row>
+    <row r="225">
+      <c r="G225" s="5" t="n"/>
+      <c r="H225" s="5" t="n"/>
+    </row>
+    <row r="226">
+      <c r="G226" s="5" t="n"/>
+      <c r="H226" s="5" t="n"/>
+    </row>
+    <row r="227">
+      <c r="G227" s="5" t="n"/>
+      <c r="H227" s="5" t="n"/>
+    </row>
+    <row r="228">
+      <c r="G228" s="5" t="n"/>
+      <c r="H228" s="5" t="n"/>
+    </row>
+    <row r="229">
+      <c r="G229" s="5" t="n"/>
+      <c r="H229" s="5" t="n"/>
+    </row>
+    <row r="230">
+      <c r="G230" s="5" t="n"/>
+      <c r="H230" s="5" t="n"/>
+    </row>
+    <row r="231">
+      <c r="G231" s="5" t="n"/>
+      <c r="H231" s="5" t="n"/>
+    </row>
+    <row r="232">
+      <c r="G232" s="5" t="n"/>
+      <c r="H232" s="5" t="n"/>
+    </row>
+    <row r="233">
+      <c r="G233" s="5" t="n"/>
+      <c r="H233" s="5" t="n"/>
+    </row>
+    <row r="234">
+      <c r="G234" s="5" t="n"/>
+      <c r="H234" s="5" t="n"/>
+    </row>
+    <row r="235">
+      <c r="G235" s="5" t="n"/>
+      <c r="H235" s="5" t="n"/>
+    </row>
+    <row r="236">
+      <c r="G236" s="5" t="n"/>
+      <c r="H236" s="5" t="n"/>
+    </row>
+    <row r="237">
+      <c r="G237" s="5" t="n"/>
+      <c r="H237" s="5" t="n"/>
+    </row>
+    <row r="238">
+      <c r="G238" s="5" t="n"/>
+      <c r="H238" s="5" t="n"/>
+    </row>
+    <row r="239">
+      <c r="G239" s="5" t="n"/>
+      <c r="H239" s="5" t="n"/>
+    </row>
+    <row r="240">
+      <c r="G240" s="5" t="n"/>
+      <c r="H240" s="5" t="n"/>
+    </row>
+    <row r="241">
+      <c r="G241" s="5" t="n"/>
+      <c r="H241" s="5" t="n"/>
+    </row>
+    <row r="242">
+      <c r="G242" s="5" t="n"/>
+      <c r="H242" s="5" t="n"/>
+    </row>
+    <row r="243">
+      <c r="G243" s="5" t="n"/>
+      <c r="H243" s="5" t="n"/>
+    </row>
+    <row r="244">
+      <c r="G244" s="5" t="n"/>
+      <c r="H244" s="5" t="n"/>
+    </row>
+    <row r="245">
+      <c r="G245" s="5" t="n"/>
+      <c r="H245" s="5" t="n"/>
+    </row>
+    <row r="246">
+      <c r="G246" s="5" t="n"/>
+      <c r="H246" s="5" t="n"/>
+    </row>
+    <row r="247">
+      <c r="G247" s="5" t="n"/>
+      <c r="H247" s="5" t="n"/>
+    </row>
+    <row r="248">
+      <c r="G248" s="5" t="n"/>
+      <c r="H248" s="5" t="n"/>
+    </row>
+    <row r="249">
+      <c r="G249" s="5" t="n"/>
+      <c r="H249" s="5" t="n"/>
+    </row>
+    <row r="250">
+      <c r="G250" s="5" t="n"/>
+      <c r="H250" s="5" t="n"/>
+    </row>
+    <row r="251">
+      <c r="G251" s="5" t="n"/>
+      <c r="H251" s="5" t="n"/>
+    </row>
+    <row r="252">
+      <c r="G252" s="5" t="n"/>
+      <c r="H252" s="5" t="n"/>
+    </row>
+    <row r="253">
+      <c r="G253" s="5" t="n"/>
+      <c r="H253" s="5" t="n"/>
+    </row>
+    <row r="254">
+      <c r="G254" s="5" t="n"/>
+      <c r="H254" s="5" t="n"/>
+    </row>
+    <row r="255">
+      <c r="G255" s="5" t="n"/>
+      <c r="H255" s="5" t="n"/>
+    </row>
+    <row r="256">
+      <c r="G256" s="5" t="n"/>
+      <c r="H256" s="5" t="n"/>
+    </row>
+    <row r="257">
+      <c r="G257" s="5" t="n"/>
+      <c r="H257" s="5" t="n"/>
+    </row>
+    <row r="258">
+      <c r="G258" s="5" t="n"/>
+      <c r="H258" s="5" t="n"/>
+    </row>
+    <row r="259">
+      <c r="G259" s="5" t="n"/>
+      <c r="H259" s="5" t="n"/>
+    </row>
+    <row r="260">
+      <c r="G260" s="5" t="n"/>
+      <c r="H260" s="5" t="n"/>
+    </row>
+    <row r="261">
+      <c r="G261" s="5" t="n"/>
+      <c r="H261" s="5" t="n"/>
+    </row>
+    <row r="262">
+      <c r="G262" s="5" t="n"/>
+      <c r="H262" s="5" t="n"/>
+    </row>
+    <row r="263">
+      <c r="G263" s="5" t="n"/>
+      <c r="H263" s="5" t="n"/>
+    </row>
+    <row r="264">
+      <c r="G264" s="5" t="n"/>
+      <c r="H264" s="5" t="n"/>
+    </row>
+    <row r="265">
+      <c r="G265" s="5" t="n"/>
+      <c r="H265" s="5" t="n"/>
+    </row>
+    <row r="266">
+      <c r="G266" s="5" t="n"/>
+      <c r="H266" s="5" t="n"/>
+    </row>
+    <row r="267">
+      <c r="G267" s="5" t="n"/>
+      <c r="H267" s="5" t="n"/>
+    </row>
+    <row r="268">
+      <c r="G268" s="5" t="n"/>
+      <c r="H268" s="5" t="n"/>
+    </row>
+    <row r="269">
+      <c r="G269" s="5" t="n"/>
+      <c r="H269" s="5" t="n"/>
+    </row>
+    <row r="270">
+      <c r="G270" s="5" t="n"/>
+      <c r="H270" s="5" t="n"/>
+    </row>
+    <row r="271">
+      <c r="G271" s="5" t="n"/>
+      <c r="H271" s="5" t="n"/>
+    </row>
+    <row r="272">
+      <c r="G272" s="5" t="n"/>
+      <c r="H272" s="5" t="n"/>
+    </row>
+    <row r="273">
+      <c r="G273" s="5" t="n"/>
+      <c r="H273" s="5" t="n"/>
+    </row>
+    <row r="274">
+      <c r="G274" s="5" t="n"/>
+      <c r="H274" s="5" t="n"/>
+    </row>
+    <row r="275">
+      <c r="G275" s="5" t="n"/>
+      <c r="H275" s="5" t="n"/>
+    </row>
+    <row r="276">
+      <c r="G276" s="5" t="n"/>
+      <c r="H276" s="5" t="n"/>
+    </row>
+    <row r="277">
+      <c r="G277" s="5" t="n"/>
+      <c r="H277" s="5" t="n"/>
+    </row>
+    <row r="278">
+      <c r="G278" s="5" t="n"/>
+      <c r="H278" s="5" t="n"/>
+    </row>
+    <row r="279">
+      <c r="G279" s="5" t="n"/>
+      <c r="H279" s="5" t="n"/>
+    </row>
+    <row r="280">
+      <c r="G280" s="5" t="n"/>
+      <c r="H280" s="5" t="n"/>
+    </row>
+    <row r="281">
+      <c r="G281" s="5" t="n"/>
+      <c r="H281" s="5" t="n"/>
+    </row>
+    <row r="282">
+      <c r="G282" s="5" t="n"/>
+      <c r="H282" s="5" t="n"/>
+    </row>
+    <row r="283">
+      <c r="G283" s="5" t="n"/>
+      <c r="H283" s="5" t="n"/>
+    </row>
+    <row r="284">
+      <c r="G284" s="5" t="n"/>
+      <c r="H284" s="5" t="n"/>
+    </row>
+    <row r="285">
+      <c r="G285" s="5" t="n"/>
+      <c r="H285" s="5" t="n"/>
+    </row>
+    <row r="286">
+      <c r="G286" s="5" t="n"/>
+      <c r="H286" s="5" t="n"/>
+    </row>
+    <row r="287">
+      <c r="G287" s="5" t="n"/>
+      <c r="H287" s="5" t="n"/>
+    </row>
+    <row r="288">
+      <c r="G288" s="5" t="n"/>
+      <c r="H288" s="5" t="n"/>
+    </row>
+    <row r="289">
+      <c r="G289" s="5" t="n"/>
+      <c r="H289" s="5" t="n"/>
+    </row>
+    <row r="290">
+      <c r="G290" s="5" t="n"/>
+      <c r="H290" s="5" t="n"/>
+    </row>
+    <row r="291">
+      <c r="G291" s="5" t="n"/>
+      <c r="H291" s="5" t="n"/>
+    </row>
+    <row r="292">
+      <c r="G292" s="5" t="n"/>
+      <c r="H292" s="5" t="n"/>
+    </row>
+    <row r="293">
+      <c r="G293" s="5" t="n"/>
+      <c r="H293" s="5" t="n"/>
+    </row>
+    <row r="294">
+      <c r="G294" s="5" t="n"/>
+      <c r="H294" s="5" t="n"/>
+    </row>
+    <row r="295">
+      <c r="G295" s="5" t="n"/>
+      <c r="H295" s="5" t="n"/>
+    </row>
+    <row r="296">
+      <c r="G296" s="5" t="n"/>
+      <c r="H296" s="5" t="n"/>
+    </row>
+    <row r="297">
+      <c r="G297" s="5" t="n"/>
+      <c r="H297" s="5" t="n"/>
+    </row>
+    <row r="298">
+      <c r="G298" s="5" t="n"/>
+      <c r="H298" s="5" t="n"/>
+    </row>
+    <row r="299">
+      <c r="G299" s="5" t="n"/>
+      <c r="H299" s="5" t="n"/>
+    </row>
+    <row r="300">
+      <c r="G300" s="5" t="n"/>
+      <c r="H300" s="5" t="n"/>
+    </row>
+    <row r="301">
+      <c r="G301" s="5" t="n"/>
+      <c r="H301" s="5" t="n"/>
+    </row>
+    <row r="302">
+      <c r="G302" s="5" t="n"/>
+      <c r="H302" s="5" t="n"/>
+    </row>
+    <row r="303">
+      <c r="G303" s="5" t="n"/>
+      <c r="H303" s="5" t="n"/>
+    </row>
+    <row r="304">
+      <c r="G304" s="5" t="n"/>
+      <c r="H304" s="5" t="n"/>
+    </row>
+    <row r="305">
+      <c r="G305" s="5" t="n"/>
+      <c r="H305" s="5" t="n"/>
+    </row>
+    <row r="306">
+      <c r="G306" s="5" t="n"/>
+      <c r="H306" s="5" t="n"/>
+    </row>
+    <row r="307">
+      <c r="G307" s="5" t="n"/>
+      <c r="H307" s="5" t="n"/>
+    </row>
+    <row r="308">
+      <c r="G308" s="5" t="n"/>
+      <c r="H308" s="5" t="n"/>
+    </row>
+    <row r="309">
+      <c r="G309" s="5" t="n"/>
+      <c r="H309" s="5" t="n"/>
+    </row>
+    <row r="310">
+      <c r="G310" s="5" t="n"/>
+      <c r="H310" s="5" t="n"/>
+    </row>
+    <row r="311">
+      <c r="G311" s="5" t="n"/>
+      <c r="H311" s="5" t="n"/>
+    </row>
+    <row r="312">
+      <c r="G312" s="5" t="n"/>
+      <c r="H312" s="5" t="n"/>
+    </row>
+    <row r="313">
+      <c r="G313" s="5" t="n"/>
+      <c r="H313" s="5" t="n"/>
+    </row>
+    <row r="314">
+      <c r="G314" s="5" t="n"/>
+      <c r="H314" s="5" t="n"/>
+    </row>
+    <row r="315">
+      <c r="G315" s="5" t="n"/>
+      <c r="H315" s="5" t="n"/>
+    </row>
+    <row r="316">
+      <c r="G316" s="5" t="n"/>
+      <c r="H316" s="5" t="n"/>
+    </row>
+    <row r="317">
+      <c r="G317" s="5" t="n"/>
+      <c r="H317" s="5" t="n"/>
+    </row>
+    <row r="318">
+      <c r="G318" s="5" t="n"/>
+      <c r="H318" s="5" t="n"/>
+    </row>
+    <row r="319">
+      <c r="G319" s="5" t="n"/>
+      <c r="H319" s="5" t="n"/>
+    </row>
+    <row r="320">
+      <c r="G320" s="5" t="n"/>
+      <c r="H320" s="5" t="n"/>
+    </row>
+    <row r="321">
+      <c r="G321" s="5" t="n"/>
+      <c r="H321" s="5" t="n"/>
+    </row>
+    <row r="322">
+      <c r="G322" s="5" t="n"/>
+      <c r="H322" s="5" t="n"/>
+    </row>
+    <row r="323">
+      <c r="G323" s="5" t="n"/>
+      <c r="H323" s="5" t="n"/>
+    </row>
+    <row r="324">
+      <c r="G324" s="5" t="n"/>
+      <c r="H324" s="5" t="n"/>
+    </row>
+    <row r="325">
+      <c r="G325" s="5" t="n"/>
+      <c r="H325" s="5" t="n"/>
+    </row>
+    <row r="326">
+      <c r="G326" s="5" t="n"/>
+      <c r="H326" s="5" t="n"/>
+    </row>
+    <row r="327">
+      <c r="G327" s="5" t="n"/>
+      <c r="H327" s="5" t="n"/>
+    </row>
+    <row r="328">
+      <c r="G328" s="5" t="n"/>
+      <c r="H328" s="5" t="n"/>
+    </row>
+    <row r="329">
+      <c r="G329" s="5" t="n"/>
+      <c r="H329" s="5" t="n"/>
+    </row>
+    <row r="330">
+      <c r="G330" s="5" t="n"/>
+      <c r="H330" s="5" t="n"/>
+    </row>
+    <row r="331">
+      <c r="G331" s="5" t="n"/>
+      <c r="H331" s="5" t="n"/>
+    </row>
+    <row r="332">
+      <c r="G332" s="5" t="n"/>
+      <c r="H332" s="5" t="n"/>
+    </row>
+    <row r="333">
+      <c r="G333" s="5" t="n"/>
+      <c r="H333" s="5" t="n"/>
+    </row>
+    <row r="334">
+      <c r="G334" s="5" t="n"/>
+      <c r="H334" s="5" t="n"/>
+    </row>
+    <row r="335">
+      <c r="G335" s="5" t="n"/>
+      <c r="H335" s="5" t="n"/>
+    </row>
+    <row r="336">
+      <c r="G336" s="5" t="n"/>
+      <c r="H336" s="5" t="n"/>
+    </row>
+    <row r="337">
+      <c r="G337" s="5" t="n"/>
+      <c r="H337" s="5" t="n"/>
+    </row>
+    <row r="338">
+      <c r="G338" s="5" t="n"/>
+      <c r="H338" s="5" t="n"/>
+    </row>
+    <row r="339">
+      <c r="G339" s="5" t="n"/>
+      <c r="H339" s="5" t="n"/>
+    </row>
+    <row r="340">
+      <c r="G340" s="5" t="n"/>
+      <c r="H340" s="5" t="n"/>
+    </row>
+    <row r="341">
+      <c r="G341" s="5" t="n"/>
+      <c r="H341" s="5" t="n"/>
+    </row>
+    <row r="342">
+      <c r="G342" s="5" t="n"/>
+      <c r="H342" s="5" t="n"/>
+    </row>
+    <row r="343">
+      <c r="G343" s="5" t="n"/>
+      <c r="H343" s="5" t="n"/>
+    </row>
+    <row r="344">
+      <c r="G344" s="5" t="n"/>
+      <c r="H344" s="5" t="n"/>
+    </row>
+    <row r="345">
+      <c r="G345" s="5" t="n"/>
+      <c r="H345" s="5" t="n"/>
+    </row>
+    <row r="346">
+      <c r="G346" s="5" t="n"/>
+      <c r="H346" s="5" t="n"/>
+    </row>
+    <row r="347">
+      <c r="G347" s="5" t="n"/>
+      <c r="H347" s="5" t="n"/>
+    </row>
+    <row r="348">
+      <c r="G348" s="5" t="n"/>
+      <c r="H348" s="5" t="n"/>
+    </row>
+    <row r="349">
+      <c r="G349" s="5" t="n"/>
+      <c r="H349" s="5" t="n"/>
+    </row>
+    <row r="350">
+      <c r="G350" s="5" t="n"/>
+      <c r="H350" s="5" t="n"/>
+    </row>
+    <row r="351">
+      <c r="G351" s="5" t="n"/>
+      <c r="H351" s="5" t="n"/>
+    </row>
+    <row r="352">
+      <c r="G352" s="5" t="n"/>
+      <c r="H352" s="5" t="n"/>
+    </row>
+    <row r="353">
+      <c r="G353" s="5" t="n"/>
+      <c r="H353" s="5" t="n"/>
+    </row>
+    <row r="354">
+      <c r="G354" s="5" t="n"/>
+      <c r="H354" s="5" t="n"/>
+    </row>
+    <row r="355">
+      <c r="G355" s="5" t="n"/>
+      <c r="H355" s="5" t="n"/>
+    </row>
+    <row r="356">
+      <c r="G356" s="5" t="n"/>
+      <c r="H356" s="5" t="n"/>
+    </row>
+    <row r="357">
+      <c r="G357" s="5" t="n"/>
+      <c r="H357" s="5" t="n"/>
+    </row>
+    <row r="358">
+      <c r="G358" s="5" t="n"/>
+      <c r="H358" s="5" t="n"/>
+    </row>
+    <row r="359">
+      <c r="G359" s="5" t="n"/>
+      <c r="H359" s="5" t="n"/>
+    </row>
+    <row r="360">
+      <c r="G360" s="5" t="n"/>
+      <c r="H360" s="5" t="n"/>
+    </row>
+    <row r="361">
+      <c r="G361" s="5" t="n"/>
+      <c r="H361" s="5" t="n"/>
+    </row>
+    <row r="362">
+      <c r="G362" s="5" t="n"/>
+      <c r="H362" s="5" t="n"/>
+    </row>
+    <row r="363">
+      <c r="G363" s="5" t="n"/>
+      <c r="H363" s="5" t="n"/>
+    </row>
+    <row r="364">
+      <c r="G364" s="5" t="n"/>
+      <c r="H364" s="5" t="n"/>
+    </row>
+    <row r="365">
+      <c r="G365" s="5" t="n"/>
+      <c r="H365" s="5" t="n"/>
+    </row>
+    <row r="366">
+      <c r="G366" s="5" t="n"/>
+      <c r="H366" s="5" t="n"/>
+    </row>
+    <row r="367">
+      <c r="G367" s="5" t="n"/>
+      <c r="H367" s="5" t="n"/>
+    </row>
+    <row r="368">
+      <c r="G368" s="5" t="n"/>
+      <c r="H368" s="5" t="n"/>
+    </row>
+    <row r="369">
+      <c r="G369" s="5" t="n"/>
+      <c r="H369" s="5" t="n"/>
+    </row>
+    <row r="370">
+      <c r="G370" s="5" t="n"/>
+      <c r="H370" s="5" t="n"/>
+    </row>
+    <row r="371">
+      <c r="G371" s="5" t="n"/>
+      <c r="H371" s="5" t="n"/>
+    </row>
+    <row r="372">
+      <c r="G372" s="5" t="n"/>
+      <c r="H372" s="5" t="n"/>
+    </row>
+    <row r="373">
+      <c r="G373" s="5" t="n"/>
+      <c r="H373" s="5" t="n"/>
+    </row>
+    <row r="374">
+      <c r="G374" s="5" t="n"/>
+      <c r="H374" s="5" t="n"/>
+    </row>
+    <row r="375">
+      <c r="G375" s="5" t="n"/>
+      <c r="H375" s="5" t="n"/>
+    </row>
+    <row r="376">
+      <c r="G376" s="5" t="n"/>
+      <c r="H376" s="5" t="n"/>
+    </row>
+    <row r="377">
+      <c r="G377" s="5" t="n"/>
+      <c r="H377" s="5" t="n"/>
+    </row>
+    <row r="378">
+      <c r="G378" s="5" t="n"/>
+      <c r="H378" s="5" t="n"/>
+    </row>
+    <row r="379">
+      <c r="G379" s="5" t="n"/>
+      <c r="H379" s="5" t="n"/>
+    </row>
+    <row r="380">
+      <c r="G380" s="5" t="n"/>
+      <c r="H380" s="5" t="n"/>
+    </row>
+    <row r="381">
+      <c r="G381" s="5" t="n"/>
+      <c r="H381" s="5" t="n"/>
+    </row>
+    <row r="382">
+      <c r="G382" s="5" t="n"/>
+      <c r="H382" s="5" t="n"/>
+    </row>
+    <row r="383">
+      <c r="G383" s="5" t="n"/>
+      <c r="H383" s="5" t="n"/>
+    </row>
+    <row r="384">
+      <c r="G384" s="5" t="n"/>
+      <c r="H384" s="5" t="n"/>
+    </row>
+    <row r="385">
+      <c r="G385" s="5" t="n"/>
+      <c r="H385" s="5" t="n"/>
+    </row>
+    <row r="386">
+      <c r="G386" s="5" t="n"/>
+      <c r="H386" s="5" t="n"/>
+    </row>
+    <row r="387">
+      <c r="G387" s="5" t="n"/>
+      <c r="H387" s="5" t="n"/>
+    </row>
+    <row r="388">
+      <c r="G388" s="5" t="n"/>
+      <c r="H388" s="5" t="n"/>
+    </row>
+    <row r="389">
+      <c r="G389" s="5" t="n"/>
+      <c r="H389" s="5" t="n"/>
+    </row>
+    <row r="390">
+      <c r="G390" s="5" t="n"/>
+      <c r="H390" s="5" t="n"/>
+    </row>
+    <row r="391">
+      <c r="G391" s="5" t="n"/>
+      <c r="H391" s="5" t="n"/>
+    </row>
+    <row r="392">
+      <c r="G392" s="5" t="n"/>
+      <c r="H392" s="5" t="n"/>
+    </row>
+    <row r="393">
+      <c r="G393" s="5" t="n"/>
+      <c r="H393" s="5" t="n"/>
+    </row>
+    <row r="394">
+      <c r="G394" s="5" t="n"/>
+      <c r="H394" s="5" t="n"/>
+    </row>
+    <row r="395">
+      <c r="G395" s="5" t="n"/>
+      <c r="H395" s="5" t="n"/>
+    </row>
+    <row r="396">
+      <c r="G396" s="5" t="n"/>
+      <c r="H396" s="5" t="n"/>
+    </row>
+    <row r="397">
+      <c r="G397" s="5" t="n"/>
+      <c r="H397" s="5" t="n"/>
+    </row>
+    <row r="398">
+      <c r="G398" s="5" t="n"/>
+      <c r="H398" s="5" t="n"/>
+    </row>
+    <row r="399">
+      <c r="G399" s="5" t="n"/>
+      <c r="H399" s="5" t="n"/>
+    </row>
+    <row r="400">
+      <c r="G400" s="5" t="n"/>
+      <c r="H400" s="5" t="n"/>
+    </row>
+    <row r="401">
+      <c r="G401" s="5" t="n"/>
+      <c r="H401" s="5" t="n"/>
+    </row>
+    <row r="402">
+      <c r="G402" s="5" t="n"/>
+      <c r="H402" s="5" t="n"/>
+    </row>
+    <row r="403">
+      <c r="G403" s="5" t="n"/>
+      <c r="H403" s="5" t="n"/>
+    </row>
+    <row r="404">
+      <c r="G404" s="5" t="n"/>
+      <c r="H404" s="5" t="n"/>
+    </row>
+    <row r="405">
+      <c r="G405" s="5" t="n"/>
+      <c r="H405" s="5" t="n"/>
+    </row>
+    <row r="406">
+      <c r="G406" s="5" t="n"/>
+      <c r="H406" s="5" t="n"/>
+    </row>
+    <row r="407">
+      <c r="G407" s="5" t="n"/>
+      <c r="H407" s="5" t="n"/>
+    </row>
+    <row r="408">
+      <c r="G408" s="5" t="n"/>
+      <c r="H408" s="5" t="n"/>
+    </row>
+    <row r="409">
+      <c r="G409" s="5" t="n"/>
+      <c r="H409" s="5" t="n"/>
+    </row>
+    <row r="410">
+      <c r="G410" s="5" t="n"/>
+      <c r="H410" s="5" t="n"/>
+    </row>
+    <row r="411">
+      <c r="G411" s="5" t="n"/>
+      <c r="H411" s="5" t="n"/>
+    </row>
+    <row r="412">
+      <c r="G412" s="5" t="n"/>
+      <c r="H412" s="5" t="n"/>
+    </row>
+    <row r="413">
+      <c r="G413" s="5" t="n"/>
+      <c r="H413" s="5" t="n"/>
+    </row>
+    <row r="414">
+      <c r="G414" s="5" t="n"/>
+      <c r="H414" s="5" t="n"/>
+    </row>
+    <row r="415">
+      <c r="G415" s="5" t="n"/>
+      <c r="H415" s="5" t="n"/>
+    </row>
+    <row r="416">
+      <c r="G416" s="5" t="n"/>
+      <c r="H416" s="5" t="n"/>
+    </row>
+    <row r="417">
+      <c r="G417" s="5" t="n"/>
+      <c r="H417" s="5" t="n"/>
+    </row>
+    <row r="418">
+      <c r="G418" s="5" t="n"/>
+      <c r="H418" s="5" t="n"/>
+    </row>
+    <row r="419">
+      <c r="G419" s="5" t="n"/>
+      <c r="H419" s="5" t="n"/>
+    </row>
+    <row r="420">
+      <c r="G420" s="5" t="n"/>
+      <c r="H420" s="5" t="n"/>
+    </row>
+    <row r="421">
+      <c r="G421" s="5" t="n"/>
+      <c r="H421" s="5" t="n"/>
+    </row>
+    <row r="422">
+      <c r="G422" s="5" t="n"/>
+      <c r="H422" s="5" t="n"/>
+    </row>
+    <row r="423">
+      <c r="G423" s="5" t="n"/>
+      <c r="H423" s="5" t="n"/>
+    </row>
+    <row r="424">
+      <c r="G424" s="5" t="n"/>
+      <c r="H424" s="5" t="n"/>
+    </row>
+    <row r="425">
+      <c r="G425" s="5" t="n"/>
+      <c r="H425" s="5" t="n"/>
+    </row>
+    <row r="426">
+      <c r="G426" s="5" t="n"/>
+      <c r="H426" s="5" t="n"/>
+    </row>
+    <row r="427">
+      <c r="G427" s="5" t="n"/>
+      <c r="H427" s="5" t="n"/>
+    </row>
+    <row r="428">
+      <c r="G428" s="5" t="n"/>
+      <c r="H428" s="5" t="n"/>
+    </row>
+    <row r="429">
+      <c r="G429" s="5" t="n"/>
+      <c r="H429" s="5" t="n"/>
+    </row>
+    <row r="430">
+      <c r="G430" s="5" t="n"/>
+      <c r="H430" s="5" t="n"/>
+    </row>
+    <row r="431">
+      <c r="G431" s="5" t="n"/>
+      <c r="H431" s="5" t="n"/>
+    </row>
+    <row r="432">
+      <c r="G432" s="5" t="n"/>
+      <c r="H432" s="5" t="n"/>
+    </row>
+    <row r="433">
+      <c r="G433" s="5" t="n"/>
+      <c r="H433" s="5" t="n"/>
+    </row>
+    <row r="434">
+      <c r="G434" s="5" t="n"/>
+      <c r="H434" s="5" t="n"/>
+    </row>
+    <row r="435">
+      <c r="G435" s="5" t="n"/>
+      <c r="H435" s="5" t="n"/>
+    </row>
+    <row r="436">
+      <c r="G436" s="5" t="n"/>
+      <c r="H436" s="5" t="n"/>
+    </row>
+    <row r="437">
+      <c r="G437" s="5" t="n"/>
+      <c r="H437" s="5" t="n"/>
+    </row>
+    <row r="438">
+      <c r="G438" s="5" t="n"/>
+      <c r="H438" s="5" t="n"/>
+    </row>
+    <row r="439">
+      <c r="G439" s="5" t="n"/>
+      <c r="H439" s="5" t="n"/>
+    </row>
+    <row r="440">
+      <c r="G440" s="5" t="n"/>
+      <c r="H440" s="5" t="n"/>
+    </row>
+    <row r="441">
+      <c r="G441" s="5" t="n"/>
+      <c r="H441" s="5" t="n"/>
+    </row>
+    <row r="442">
+      <c r="G442" s="5" t="n"/>
+      <c r="H442" s="5" t="n"/>
+    </row>
+    <row r="443">
+      <c r="G443" s="5" t="n"/>
+      <c r="H443" s="5" t="n"/>
+    </row>
+    <row r="444">
+      <c r="G444" s="5" t="n"/>
+      <c r="H444" s="5" t="n"/>
+    </row>
+    <row r="445">
+      <c r="G445" s="5" t="n"/>
+      <c r="H445" s="5" t="n"/>
+    </row>
+    <row r="446">
+      <c r="G446" s="5" t="n"/>
+      <c r="H446" s="5" t="n"/>
+    </row>
+    <row r="447">
+      <c r="G447" s="5" t="n"/>
+      <c r="H447" s="5" t="n"/>
+    </row>
+    <row r="448">
+      <c r="G448" s="5" t="n"/>
+      <c r="H448" s="5" t="n"/>
+    </row>
+    <row r="449">
+      <c r="G449" s="5" t="n"/>
+      <c r="H449" s="5" t="n"/>
+    </row>
+    <row r="450">
+      <c r="G450" s="5" t="n"/>
+      <c r="H450" s="5" t="n"/>
+    </row>
+    <row r="451">
+      <c r="G451" s="5" t="n"/>
+      <c r="H451" s="5" t="n"/>
+    </row>
+    <row r="452">
+      <c r="G452" s="5" t="n"/>
+      <c r="H452" s="5" t="n"/>
+    </row>
+    <row r="453">
+      <c r="G453" s="5" t="n"/>
+      <c r="H453" s="5" t="n"/>
+    </row>
+    <row r="454">
+      <c r="G454" s="5" t="n"/>
+      <c r="H454" s="5" t="n"/>
+    </row>
+    <row r="455">
+      <c r="G455" s="5" t="n"/>
+      <c r="H455" s="5" t="n"/>
+    </row>
+    <row r="456">
+      <c r="G456" s="5" t="n"/>
+      <c r="H456" s="5" t="n"/>
+    </row>
+    <row r="457">
+      <c r="G457" s="5" t="n"/>
+      <c r="H457" s="5" t="n"/>
+    </row>
+    <row r="458">
+      <c r="G458" s="5" t="n"/>
+      <c r="H458" s="5" t="n"/>
+    </row>
+    <row r="459">
+      <c r="G459" s="5" t="n"/>
+      <c r="H459" s="5" t="n"/>
+    </row>
+    <row r="460">
+      <c r="G460" s="5" t="n"/>
+      <c r="H460" s="5" t="n"/>
+    </row>
+    <row r="461">
+      <c r="G461" s="5" t="n"/>
+      <c r="H461" s="5" t="n"/>
+    </row>
+    <row r="462">
+      <c r="G462" s="5" t="n"/>
+      <c r="H462" s="5" t="n"/>
+    </row>
+    <row r="463">
+      <c r="G463" s="5" t="n"/>
+      <c r="H463" s="5" t="n"/>
+    </row>
+    <row r="464">
+      <c r="G464" s="5" t="n"/>
+      <c r="H464" s="5" t="n"/>
+    </row>
+    <row r="465">
+      <c r="G465" s="5" t="n"/>
+      <c r="H465" s="5" t="n"/>
+    </row>
+    <row r="466">
+      <c r="G466" s="5" t="n"/>
+      <c r="H466" s="5" t="n"/>
+    </row>
+    <row r="467">
+      <c r="G467" s="5" t="n"/>
+      <c r="H467" s="5" t="n"/>
+    </row>
+    <row r="468">
+      <c r="G468" s="5" t="n"/>
+      <c r="H468" s="5" t="n"/>
+    </row>
+    <row r="469">
+      <c r="G469" s="5" t="n"/>
+      <c r="H469" s="5" t="n"/>
+    </row>
+    <row r="470">
+      <c r="G470" s="5" t="n"/>
+      <c r="H470" s="5" t="n"/>
+    </row>
+    <row r="471">
+      <c r="G471" s="5" t="n"/>
+      <c r="H471" s="5" t="n"/>
+    </row>
+    <row r="472">
+      <c r="G472" s="5" t="n"/>
+      <c r="H472" s="5" t="n"/>
+    </row>
+    <row r="473">
+      <c r="G473" s="5" t="n"/>
+      <c r="H473" s="5" t="n"/>
+    </row>
+    <row r="474">
+      <c r="G474" s="5" t="n"/>
+      <c r="H474" s="5" t="n"/>
+    </row>
+    <row r="475">
+      <c r="G475" s="5" t="n"/>
+      <c r="H475" s="5" t="n"/>
+    </row>
+    <row r="476">
+      <c r="G476" s="5" t="n"/>
+      <c r="H476" s="5" t="n"/>
+    </row>
+    <row r="477">
+      <c r="G477" s="5" t="n"/>
+      <c r="H477" s="5" t="n"/>
+    </row>
+    <row r="478">
+      <c r="G478" s="5" t="n"/>
+      <c r="H478" s="5" t="n"/>
+    </row>
+    <row r="479">
+      <c r="G479" s="5" t="n"/>
+      <c r="H479" s="5" t="n"/>
+    </row>
+    <row r="480">
+      <c r="G480" s="5" t="n"/>
+      <c r="H480" s="5" t="n"/>
+    </row>
+    <row r="481">
+      <c r="G481" s="5" t="n"/>
+      <c r="H481" s="5" t="n"/>
+    </row>
+    <row r="482">
+      <c r="G482" s="5" t="n"/>
+      <c r="H482" s="5" t="n"/>
+    </row>
+    <row r="483">
+      <c r="G483" s="5" t="n"/>
+      <c r="H483" s="5" t="n"/>
+    </row>
+    <row r="484">
+      <c r="G484" s="5" t="n"/>
+      <c r="H484" s="5" t="n"/>
+    </row>
+    <row r="485">
+      <c r="G485" s="5" t="n"/>
+      <c r="H485" s="5" t="n"/>
+    </row>
+    <row r="486">
+      <c r="G486" s="5" t="n"/>
+      <c r="H486" s="5" t="n"/>
+    </row>
+    <row r="487">
+      <c r="G487" s="5" t="n"/>
+      <c r="H487" s="5" t="n"/>
+    </row>
+    <row r="488">
+      <c r="G488" s="5" t="n"/>
+      <c r="H488" s="5" t="n"/>
+    </row>
+    <row r="489">
+      <c r="G489" s="5" t="n"/>
+      <c r="H489" s="5" t="n"/>
+    </row>
+    <row r="490">
+      <c r="G490" s="5" t="n"/>
+      <c r="H490" s="5" t="n"/>
+    </row>
+    <row r="491">
+      <c r="G491" s="5" t="n"/>
+      <c r="H491" s="5" t="n"/>
+    </row>
+    <row r="492">
+      <c r="G492" s="5" t="n"/>
+      <c r="H492" s="5" t="n"/>
+    </row>
+    <row r="493">
+      <c r="G493" s="5" t="n"/>
+      <c r="H493" s="5" t="n"/>
+    </row>
+    <row r="494">
+      <c r="G494" s="5" t="n"/>
+      <c r="H494" s="5" t="n"/>
+    </row>
+    <row r="495">
+      <c r="G495" s="5" t="n"/>
+      <c r="H495" s="5" t="n"/>
+    </row>
+    <row r="496">
+      <c r="G496" s="5" t="n"/>
+      <c r="H496" s="5" t="n"/>
+    </row>
+    <row r="497">
+      <c r="G497" s="5" t="n"/>
+      <c r="H497" s="5" t="n"/>
+    </row>
+    <row r="498">
+      <c r="G498" s="5" t="n"/>
+      <c r="H498" s="5" t="n"/>
+    </row>
+    <row r="499">
+      <c r="G499" s="5" t="n"/>
+      <c r="H499" s="5" t="n"/>
+    </row>
+    <row r="500">
+      <c r="G500" s="5" t="n"/>
+      <c r="H500" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>